<commit_message>
added isotherm input function, fixed units for Excel files which I only included dimensions unit, kept all breakthrough data and parameters in one file
</commit_message>
<xml_diff>
--- a/src/reactormodels/IO/data/experimental_input_breakthrough.xlsx
+++ b/src/reactormodels/IO/data/experimental_input_breakthrough.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mohammedfaran/Desktop/python_models/ReactorModels/src/reactormodels/IO/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9FB707-D1C4-4149-8A55-1D9EB029F39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6098BB76-96BC-1143-BA90-3AC250894255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1720" yWindow="1480" windowWidth="26700" windowHeight="15940" xr2:uid="{BEB422E4-985B-DA42-A0EA-C89047788836}"/>
+    <workbookView xWindow="2100" yWindow="1760" windowWidth="26700" windowHeight="15940" xr2:uid="{BEB422E4-985B-DA42-A0EA-C89047788836}"/>
   </bookViews>
   <sheets>
-    <sheet name="feed_concentration" sheetId="1" r:id="rId1"/>
-    <sheet name="effluent_concentration" sheetId="2" r:id="rId2"/>
-    <sheet name="initial_concentration" sheetId="4" r:id="rId3"/>
-    <sheet name="notes" sheetId="3" r:id="rId4"/>
+    <sheet name="breakthrough_parameters" sheetId="5" r:id="rId1"/>
+    <sheet name="feed_concentration" sheetId="1" r:id="rId2"/>
+    <sheet name="effluent_concentration" sheetId="2" r:id="rId3"/>
+    <sheet name="initial_concentration" sheetId="4" r:id="rId4"/>
+    <sheet name="notes" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
   <si>
     <t xml:space="preserve">time </t>
   </si>
@@ -67,6 +68,36 @@
   <si>
     <t>4:2 FTS</t>
   </si>
+  <si>
+    <t>breakthrough</t>
+  </si>
+  <si>
+    <t>parameters</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>flow_rate</t>
+  </si>
+  <si>
+    <t>superficial_velocity</t>
+  </si>
+  <si>
+    <t>initial_mass_fraction</t>
+  </si>
+  <si>
+    <t>[L^3/t]</t>
+  </si>
+  <si>
+    <t>[M/M]</t>
+  </si>
+  <si>
+    <t>[L/t]</t>
+  </si>
 </sst>
 </file>
 
@@ -77,7 +108,7 @@
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -112,8 +143,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -126,8 +164,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -150,12 +194,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -164,6 +245,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -498,6 +592,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28273D33-CC04-8B4C-B07E-FF186E451A94}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="14"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="9">
+        <v>9.6333299999999996E-8</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="10">
+        <v>1.213E-2</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC90306C-9E69-C147-806A-A4F4F1854575}">
   <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1968,7 +2127,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{895A8352-4055-1E44-A64F-1E17485D6E3F}">
   <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3439,7 +3598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A762BF2D-9395-A948-9B93-3EB16D030FFC}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3508,7 +3667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E47A9B8-725A-0F4C-A7BB-A7D31C9058DC}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>